<commit_message>
Initial commit: Elevator Automation System TIA Portal v19
</commit_message>
<xml_diff>
--- a/Mechs.xlsx
+++ b/Mechs.xlsx
@@ -2,26 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Constants" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="TagTable Properties" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
+      <loext:extCalcPr stringRefSyntax="CalcA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="27">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -47,31 +46,61 @@
     <t xml:space="preserve">UInt</t>
   </si>
   <si>
-    <t xml:space="preserve">кількість реальних пристроїв </t>
+    <t xml:space="preserve">Верхня межа масиву Gate2P[] (кількість засувок - 1)</t>
   </si>
   <si>
     <t xml:space="preserve">REDLERS_COUNT</t>
   </si>
   <si>
+    <t xml:space="preserve">Верхня межа масиву Redler[] (кількість редлерів - 1)</t>
+  </si>
+  <si>
     <t xml:space="preserve">NORIAS_COUNT</t>
   </si>
   <si>
-    <t xml:space="preserve">0</t>
+    <t xml:space="preserve">Верхня межа масиву Noria[] (кількість норій - 1)</t>
   </si>
   <si>
     <t xml:space="preserve">FANS_COUNT</t>
   </si>
   <si>
+    <t xml:space="preserve">Верхня межа масиву Fan[] (кількість вентиляторів - 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RECEIVING_PITS_COUNT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Верхня межа масиву ReceivingPit[] (кількість приймальних ям - 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEPARATORS_COUNT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Верхня межа масиву Separator[] (кількість сепараторів - 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALVES3P_COUNT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Верхня межа масиву Valve3P[] (кількість клапанів 3П - 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SILOS_COUNT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Верхня межа масиву Silos[] (кількість силосів - 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUSHKAS_COUNT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Верхня межа масиву Sushka[] (кількість сушарок - 1)</t>
+  </si>
+  <si>
     <t xml:space="preserve">MECHS_COUNT</t>
   </si>
   <si>
-    <t xml:space="preserve">сума кількості всих механізмів </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BelongsToUnit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accessibility</t>
+    <t xml:space="preserve">Верхня межа масиву Mechs[] (max SlotId серед усіх пристроїв)</t>
   </si>
 </sst>
 </file>
@@ -83,10 +112,10 @@
   </numFmts>
   <fonts count="4">
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <sz val="10"/>
@@ -154,7 +183,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -281,10 +310,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="57.4"/>
+  </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -301,7 +337,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -312,13 +348,13 @@
         <v>7</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>3</v>
+        <v>80</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -329,107 +365,155 @@
         <v>7</v>
       </c>
       <c r="D3" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>14</v>
+      <c r="E10" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>313</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+    <oddHeader>&amp;C&amp;"Times New Roman,Звичайний"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Звичайний"&amp;12Сторінка &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>